<commit_message>
ran weighting analysis (besides sensitivity analysis)
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/entropy_weights.xlsx
+++ b/Scoring Logic and Documentation/method/entropy_weights.xlsx
@@ -478,28 +478,28 @@
         <v>0.3</v>
       </c>
       <c r="C2" t="n">
-        <v>0.237202641363488</v>
+        <v>0.2077009794300993</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3906803210429771</v>
+        <v>0.3329873688719885</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09531178634326594</v>
+        <v>0.0940213799053623</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2852135684465159</v>
+        <v>0.2796442862775838</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06279735863651195</v>
+        <v>0.09229902056990072</v>
       </c>
       <c r="H2" t="n">
-        <v>0.09068032104297713</v>
+        <v>0.0329873688719885</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2046882136567341</v>
+        <v>0.2059786200946377</v>
       </c>
       <c r="J2" t="n">
-        <v>0.01478643155348414</v>
+        <v>0.02035571372241624</v>
       </c>
     </row>
     <row r="3">
@@ -512,28 +512,28 @@
         <v>0.35</v>
       </c>
       <c r="C3" t="n">
-        <v>0.375533028403626</v>
+        <v>0.3657095993362007</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3639991243790874</v>
+        <v>0.3175616523168405</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5367557442735834</v>
+        <v>0.528644628220389</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1406130186775549</v>
+        <v>0.1368173462482312</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02553302840362598</v>
+        <v>0.0157095993362007</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0139991243790874</v>
+        <v>0.03243834768315945</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1867557442735834</v>
+        <v>0.1786446282203891</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2093869813224451</v>
+        <v>0.2131826537517688</v>
       </c>
     </row>
     <row r="4">
@@ -546,28 +546,28 @@
         <v>0.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1695405999026638</v>
+        <v>0.1937021285305291</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2065014145762053</v>
+        <v>0.2743280127150262</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1360412431314365</v>
+        <v>0.1400228069035754</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2135483537345129</v>
+        <v>0.2086676978377357</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03045940009733616</v>
+        <v>0.006297871469470945</v>
       </c>
       <c r="H4" t="n">
-        <v>0.006501414576205261</v>
+        <v>0.0743280127150262</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0639587568685635</v>
+        <v>0.05997719309642463</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01354835373451285</v>
+        <v>0.008667697837735716</v>
       </c>
     </row>
     <row r="5">
@@ -580,28 +580,28 @@
         <v>0.15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2177237303302222</v>
+        <v>0.232887292703171</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03881914000173024</v>
+        <v>0.0751229660961448</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2318912262517141</v>
+        <v>0.2373111849706733</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3606250591414165</v>
+        <v>0.3748706696364494</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06772373033022216</v>
+        <v>0.08288729270317097</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1111808599982698</v>
+        <v>0.07487703390385519</v>
       </c>
       <c r="I5" t="n">
-        <v>0.08189122625171411</v>
+        <v>0.08731118497067328</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2106250591414165</v>
+        <v>0.2248706696364494</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
massive cleaning refactor +sensitivity analysis ran
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/entropy_weights.xlsx
+++ b/Scoring Logic and Documentation/method/entropy_weights.xlsx
@@ -478,28 +478,28 @@
         <v>0.3</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2077009794300993</v>
+        <v>0.2682983388297028</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3329873688719885</v>
+        <v>0.3364509052363785</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0940213799053623</v>
+        <v>0.1931820745121725</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2796442862775838</v>
+        <v>0.3336114288123433</v>
       </c>
       <c r="G2" t="n">
-        <v>0.09229902056990072</v>
+        <v>0.03170166117029721</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0329873688719885</v>
+        <v>0.03645090523637851</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2059786200946377</v>
+        <v>0.1068179254878275</v>
       </c>
       <c r="J2" t="n">
-        <v>0.02035571372241624</v>
+        <v>0.03361142881234336</v>
       </c>
     </row>
     <row r="3">
@@ -512,28 +512,28 @@
         <v>0.35</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3657095993362007</v>
+        <v>0.3705150512541915</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3175616523168405</v>
+        <v>0.3203795033433237</v>
       </c>
       <c r="E3" t="n">
-        <v>0.528644628220389</v>
+        <v>0.4651563417489527</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1368173462482312</v>
+        <v>0.3139687993512856</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0157095993362007</v>
+        <v>0.02051505125419151</v>
       </c>
       <c r="H3" t="n">
-        <v>0.03243834768315945</v>
+        <v>0.02962049665667627</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1786446282203891</v>
+        <v>0.1151563417489527</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2131826537517688</v>
+        <v>0.03603120064871435</v>
       </c>
     </row>
     <row r="4">
@@ -546,28 +546,28 @@
         <v>0.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1937021285305291</v>
+        <v>0.16268896692254</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2743280127150262</v>
+        <v>0.2694864993731558</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1400228069035754</v>
+        <v>0.1236147136516962</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2086676978377357</v>
+        <v>0.1265816336234309</v>
       </c>
       <c r="G4" t="n">
-        <v>0.006297871469470945</v>
+        <v>0.03731103307745998</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0743280127150262</v>
+        <v>0.06948649937315576</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05997719309642463</v>
+        <v>0.07638528634830379</v>
       </c>
       <c r="J4" t="n">
-        <v>0.008667697837735716</v>
+        <v>0.07341836637656907</v>
       </c>
     </row>
     <row r="5">
@@ -580,28 +580,28 @@
         <v>0.15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.232887292703171</v>
+        <v>0.1984976429935657</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0751229660961448</v>
+        <v>0.07368309204714199</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2373111849706733</v>
+        <v>0.2180468700871786</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3748706696364494</v>
+        <v>0.22583813821294</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08288729270317097</v>
+        <v>0.04849764299356571</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07487703390385519</v>
+        <v>0.076316907952858</v>
       </c>
       <c r="I5" t="n">
-        <v>0.08731118497067328</v>
+        <v>0.06804687008717861</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2248706696364494</v>
+        <v>0.07583813821294005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate entropy/MEREC weights on the new ground truth; fix merec_weights output path
merec_weights.py resolved its output and GT search dirs from the script folder
(Miscellaneous Scripts/...), so it wrote to a stray folder; both now use PROJECT_ROOT.
SensitivityAnalysis.py's typed-in per-type vectors match the new Table S2.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AwjALCmxts3WuvoDW8hNtv
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/entropy_weights.xlsx
+++ b/Scoring Logic and Documentation/method/entropy_weights.xlsx
@@ -478,28 +478,28 @@
         <v>0.3</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2686826806918144</v>
+        <v>0.2724233791491785</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3364509052363785</v>
+        <v>0.3373637073689004</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1931820745121725</v>
+        <v>0.1904603094003465</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3353560355741635</v>
+        <v>0.3332241012030146</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03131731930818554</v>
+        <v>0.02757662085082152</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03645090523637851</v>
+        <v>0.03736370736890043</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1068179254878275</v>
+        <v>0.1095396905996535</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0353560355741635</v>
+        <v>0.03322410120301461</v>
       </c>
     </row>
     <row r="3">
@@ -512,28 +512,28 @@
         <v>0.35</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3710458202681205</v>
+        <v>0.3701337959499669</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3203795033433237</v>
+        <v>0.3148134821932385</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4651563417489527</v>
+        <v>0.4667255263970893</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3156106858187211</v>
+        <v>0.3181531880446986</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02104582026812052</v>
+        <v>0.02013379594996689</v>
       </c>
       <c r="H3" t="n">
-        <v>0.02962049665667627</v>
+        <v>0.03518651780676152</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1151563417489527</v>
+        <v>0.1167255263970893</v>
       </c>
       <c r="J3" t="n">
-        <v>0.03438931418127888</v>
+        <v>0.03184681195530137</v>
       </c>
     </row>
     <row r="4">
@@ -546,28 +546,28 @@
         <v>0.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1614895048497469</v>
+        <v>0.171469134070057</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2694864993731558</v>
+        <v>0.2776395167198066</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1236147136516962</v>
+        <v>0.1240317225012729</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1220141294665648</v>
+        <v>0.1229970530800816</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03851049515025309</v>
+        <v>0.02853086592994297</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06948649937315576</v>
+        <v>0.07763951671980657</v>
       </c>
       <c r="I4" t="n">
-        <v>0.07638528634830379</v>
+        <v>0.07596827749872707</v>
       </c>
       <c r="J4" t="n">
-        <v>0.07798587053343521</v>
+        <v>0.07700294691991842</v>
       </c>
     </row>
     <row r="5">
@@ -580,28 +580,28 @@
         <v>0.15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1987819941903182</v>
+        <v>0.1859736908307976</v>
       </c>
       <c r="D5" t="n">
-        <v>0.07368309204714199</v>
+        <v>0.07018329371805455</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2180468700871786</v>
+        <v>0.2187824417012913</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2270191491405506</v>
+        <v>0.2256256576722052</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04878199419031817</v>
+        <v>0.0359736908307976</v>
       </c>
       <c r="H5" t="n">
-        <v>0.076316907952858</v>
+        <v>0.07981670628194544</v>
       </c>
       <c r="I5" t="n">
-        <v>0.06804687008717861</v>
+        <v>0.0687824417012913</v>
       </c>
       <c r="J5" t="n">
-        <v>0.07701914914055064</v>
+        <v>0.07562565767220519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>